<commit_message>
feat(security): SEC-17 — shade placeholder rows (FCE4D6) in the six delivery workbooks, security_v11
</commit_message>
<xml_diff>
--- a/features/security/sandbox/delivery/FM-WI-FSM-036-A01 STLA 測試用例規範與結果_SWQT STLA Test Case Specification & Result_SWQT_Security_CertProvider_20260917.xlsx
+++ b/features/security/sandbox/delivery/FM-WI-FSM-036-A01 STLA 測試用例規範與結果_SWQT STLA Test Case Specification & Result_SWQT_Security_CertProvider_20260917.xlsx
@@ -4228,7 +4228,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -4268,6 +4268,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF002060"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE4D6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -4896,7 +4902,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="176">
+  <cellXfs count="183">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="8" applyBorder="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="8" applyBorder="1"/>
@@ -5381,6 +5387,23 @@
     <xf numFmtId="0" fontId="43" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf fillId="8" applyFill="1" numFmtId="0" fontId="0" borderId="0" xfId="0"/>
+    <xf fillId="8" applyFill="1" numFmtId="0" fontId="56" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf fillId="8" applyFill="1" numFmtId="0" fontId="56" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fillId="8" applyFill="1" numFmtId="0" fontId="56" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf fillId="8" applyFill="1" numFmtId="0" fontId="56" borderId="45" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fillId="8" applyFill="1" numFmtId="0" fontId="55" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf fillId="8" applyFill="1" numFmtId="0" fontId="56" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="19">
     <cellStyle name="Normal 2 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -8072,52 +8095,52 @@
       </c>
     </row>
     <row r="11" spans="1:34" s="84" customFormat="1">
-      <c r="A11" s="80"/>
-      <c r="B11" s="81" t="str">
+      <c r="A11" s="177"/>
+      <c r="B11" s="178" t="str">
         <f t="shared" ref="B11:B74" si="0">IF(ISBLANK($D11),"",ROW()-9)</f>
         <v/>
       </c>
-      <c r="C11" s="82"/>
-      <c r="D11" s="81" t="inlineStr">
+      <c r="C11" s="179"/>
+      <c r="D11" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">SWE1-CertProvider-001</t>
         </is>
       </c>
-      <c r="E11" s="81"/>
-      <c r="F11" s="81" t="inlineStr">
+      <c r="E11" s="178"/>
+      <c r="F11" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NR1L-CP-002</t>
         </is>
       </c>
-      <c r="G11" s="81" t="inlineStr">
+      <c r="G11" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">Cert Provider</t>
         </is>
       </c>
-      <c r="H11" s="81" t="inlineStr">
+      <c r="H11" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">Chain Verification</t>
         </is>
       </c>
-      <c r="I11" s="81" t="inlineStr">
+      <c r="I11" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">The Cert Provider feature shall verify the integrity and authenticity of an X.509 leaf certificate provided by an external application.
 (broken certificate chain; verification is rejected)</t>
         </is>
       </c>
-      <c r="J11" s="81" t="inlineStr">
+      <c r="J11" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. DUT is connected via ADB with root permission (Dev/Eng build)
 2. Test runner CertProviderAndroidInstrumentalTest.apk is installed
 3. Certificate assets are available under SecurityAssets/oem-certs/cert-provider/</t>
         </is>
       </c>
-      <c r="K11" s="81" t="inlineStr">
+      <c r="K11" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NA</t>
         </is>
       </c>
-      <c r="L11" s="81" t="inlineStr">
+      <c r="L11" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. Run the OpenSSL chain verification of the certificate on the host
 $ openssl verify -verbose -CAfile RootCert.pem -untrusted L1.pem -untrusted L2.pem -untrusted L3.pem SAMcert.pem
@@ -8127,86 +8150,86 @@
 $ adb logcat -s MelcoCertProviderTest</t>
         </is>
       </c>
-      <c r="M11" s="81" t="inlineStr">
+      <c r="M11" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. The openssl command prints "unable to get issuer certificate" on stdout
 2. The instrumentation runner reports "OK (1 test)" for fotaMcpuCertTestBrokenCert
 3. &lt;log keyword provided by RD (X-h)&gt;</t>
         </is>
       </c>
-      <c r="N11" s="81" t="inlineStr">
+      <c r="N11" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-001</t>
         </is>
       </c>
-      <c r="O11" s="81" t="inlineStr">
+      <c r="O11" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NEW</t>
         </is>
       </c>
-      <c r="P11" s="81" t="inlineStr">
+      <c r="P11" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">P0</t>
         </is>
       </c>
-      <c r="Q11" s="81"/>
-      <c r="R11" s="81" t="inlineStr">
+      <c r="Q11" s="178"/>
+      <c r="R11" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">負向測試 (Negative / Invalid)</t>
         </is>
       </c>
-      <c r="S11" s="81" t="inlineStr">
+      <c r="S11" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">No</t>
         </is>
       </c>
-      <c r="T11" s="81" t="inlineStr">
+      <c r="T11" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="U11" s="81" t="inlineStr">
+      <c r="U11" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="V11" s="81" t="inlineStr">
+      <c r="V11" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="W11" s="81" t="inlineStr">
+      <c r="W11" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="X11" s="83" t="inlineStr">
+      <c r="X11" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="Y11" s="81" t="inlineStr">
+      <c r="Y11" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="Z11" s="83" t="inlineStr">
+      <c r="Z11" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="AA11" s="83" t="inlineStr">
+      <c r="AA11" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">PeiPYHsu</t>
         </is>
       </c>
-      <c r="AB11" s="81"/>
-      <c r="AC11" s="81"/>
-      <c r="AD11" s="81"/>
-      <c r="AE11" s="81"/>
-      <c r="AF11" s="81"/>
-      <c r="AG11" s="81"/>
-      <c r="AH11" s="83" t="inlineStr">
+      <c r="AB11" s="178"/>
+      <c r="AC11" s="178"/>
+      <c r="AD11" s="178"/>
+      <c r="AE11" s="178"/>
+      <c r="AF11" s="178"/>
+      <c r="AG11" s="178"/>
+      <c r="AH11" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">source: 037 SWE1-CertProvider-001 Requirement Description and Verification Criteria
 Polarion: NRL-349384
@@ -8365,40 +8388,40 @@
       </c>
     </row>
     <row r="13" spans="1:34">
-      <c r="A13" s="87"/>
-      <c r="B13" s="81" t="str">
+      <c r="A13" s="182"/>
+      <c r="B13" s="178" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="C13" s="82"/>
-      <c r="D13" s="81" t="inlineStr">
+      <c r="C13" s="179"/>
+      <c r="D13" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">SWE1-CertProvider-002</t>
         </is>
       </c>
-      <c r="E13" s="81"/>
-      <c r="F13" s="81" t="inlineStr">
+      <c r="E13" s="178"/>
+      <c r="F13" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NR1L-CP-004</t>
         </is>
       </c>
-      <c r="G13" s="81" t="inlineStr">
+      <c r="G13" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">Cert Provider</t>
         </is>
       </c>
-      <c r="H13" s="81" t="inlineStr">
+      <c r="H13" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">Field Matching</t>
         </is>
       </c>
-      <c r="I13" s="81" t="inlineStr">
+      <c r="I13" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">The Cert Provider feature shall verify that the Subject field of the leaf certificate matches the expected value defined in the configuration or provided dynamically.
 (subject name not identical to the configuration; certificate is rejected)</t>
         </is>
       </c>
-      <c r="J13" s="81" t="inlineStr">
+      <c r="J13" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. DUT is connected via ADB with root permission (Dev/Eng build)
 2. Test runner CertProviderAndroidInstrumentalTest.apk is installed
@@ -8406,12 +8429,12 @@
 4. Configuration files are available under SecurityAssets/oem-certs/cert-provider/{TYPE}/cfgs/</t>
         </is>
       </c>
-      <c r="K13" s="81" t="inlineStr">
+      <c r="K13" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NA</t>
         </is>
       </c>
-      <c r="L13" s="81" t="inlineStr">
+      <c r="L13" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. Read the Subject field of the certificate on the host
 $ openssl x509 -in leaf.crt -text
@@ -8421,86 +8444,86 @@
 $ &lt;command provided by RD (X-e)&gt;</t>
         </is>
       </c>
-      <c r="M13" s="81" t="inlineStr">
+      <c r="M13" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. The openssl x509 output shows a "Subject:" line that is not identical to the subject name in SecurityAssets/oem-certs/cert-provider/{TYPE}/cfgs/
 2. The openssl command prints "SAMcert.pem: OK" on stdout
 3. &lt;log keyword provided by RD (X-h)&gt;</t>
         </is>
       </c>
-      <c r="N13" s="81" t="inlineStr">
+      <c r="N13" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-002</t>
         </is>
       </c>
-      <c r="O13" s="81" t="inlineStr">
+      <c r="O13" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NEW</t>
         </is>
       </c>
-      <c r="P13" s="81" t="inlineStr">
+      <c r="P13" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">P1</t>
         </is>
       </c>
-      <c r="Q13" s="81"/>
-      <c r="R13" s="81" t="inlineStr">
+      <c r="Q13" s="178"/>
+      <c r="R13" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">負向測試 (Negative / Invalid)</t>
         </is>
       </c>
-      <c r="S13" s="81" t="inlineStr">
+      <c r="S13" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">No</t>
         </is>
       </c>
-      <c r="T13" s="81" t="inlineStr">
+      <c r="T13" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="U13" s="81" t="inlineStr">
+      <c r="U13" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="V13" s="81" t="inlineStr">
+      <c r="V13" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="W13" s="81" t="inlineStr">
+      <c r="W13" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="X13" s="83" t="inlineStr">
+      <c r="X13" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="Y13" s="81" t="inlineStr">
+      <c r="Y13" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="Z13" s="83" t="inlineStr">
+      <c r="Z13" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="AA13" s="83" t="inlineStr">
+      <c r="AA13" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">PeiPYHsu</t>
         </is>
       </c>
-      <c r="AB13" s="81"/>
-      <c r="AC13" s="81"/>
-      <c r="AD13" s="81"/>
-      <c r="AE13" s="81"/>
-      <c r="AF13" s="81"/>
-      <c r="AG13" s="81"/>
-      <c r="AH13" s="83" t="inlineStr">
+      <c r="AB13" s="178"/>
+      <c r="AC13" s="178"/>
+      <c r="AD13" s="178"/>
+      <c r="AE13" s="178"/>
+      <c r="AF13" s="178"/>
+      <c r="AG13" s="178"/>
+      <c r="AH13" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">source: 037 SWE1-CertProvider-002 Requirement Description and Verification Criteria
 Polarion: NRL-349385
@@ -8659,40 +8682,40 @@
       </c>
     </row>
     <row r="15" spans="1:34">
-      <c r="A15" s="87"/>
-      <c r="B15" s="81" t="str">
+      <c r="A15" s="182"/>
+      <c r="B15" s="178" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="C15" s="82"/>
-      <c r="D15" s="81" t="inlineStr">
+      <c r="C15" s="179"/>
+      <c r="D15" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">SWE1-CertProvider-003</t>
         </is>
       </c>
-      <c r="E15" s="81"/>
-      <c r="F15" s="81" t="inlineStr">
+      <c r="E15" s="178"/>
+      <c r="F15" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NR1L-CP-006</t>
         </is>
       </c>
-      <c r="G15" s="81" t="inlineStr">
+      <c r="G15" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">Cert Provider</t>
         </is>
       </c>
-      <c r="H15" s="81" t="inlineStr">
+      <c r="H15" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">Field Matching</t>
         </is>
       </c>
-      <c r="I15" s="81" t="inlineStr">
+      <c r="I15" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">The Cert Provider feature shall verify that the Issuer field of the leaf certificate matches the expected value defined in the configuration.
 (issuer name not identical to the configuration; certificate is rejected)</t>
         </is>
       </c>
-      <c r="J15" s="81" t="inlineStr">
+      <c r="J15" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. DUT is connected via ADB with root permission (Dev/Eng build)
 2. Test runner CertProviderAndroidInstrumentalTest.apk is installed
@@ -8700,12 +8723,12 @@
 4. Configuration files are available under SecurityAssets/oem-certs/cert-provider/{TYPE}/cfgs/</t>
         </is>
       </c>
-      <c r="K15" s="81" t="inlineStr">
+      <c r="K15" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NA</t>
         </is>
       </c>
-      <c r="L15" s="81" t="inlineStr">
+      <c r="L15" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. Read the Issuer field of the certificate on the host
 $ openssl x509 -in leaf.crt -text
@@ -8715,86 +8738,86 @@
 $ &lt;command provided by RD (X-e)&gt;</t>
         </is>
       </c>
-      <c r="M15" s="81" t="inlineStr">
+      <c r="M15" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. The openssl x509 output shows an "Issuer:" line that is not identical to the issuer name in SecurityAssets/oem-certs/cert-provider/{TYPE}/cfgs/
 2. The openssl command prints "SAMcert.pem: OK" on stdout
 3. &lt;log keyword provided by RD (X-h)&gt;</t>
         </is>
       </c>
-      <c r="N15" s="81" t="inlineStr">
+      <c r="N15" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-003</t>
         </is>
       </c>
-      <c r="O15" s="81" t="inlineStr">
+      <c r="O15" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NEW</t>
         </is>
       </c>
-      <c r="P15" s="81" t="inlineStr">
+      <c r="P15" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">P1</t>
         </is>
       </c>
-      <c r="Q15" s="81"/>
-      <c r="R15" s="81" t="inlineStr">
+      <c r="Q15" s="178"/>
+      <c r="R15" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">負向測試 (Negative / Invalid)</t>
         </is>
       </c>
-      <c r="S15" s="81" t="inlineStr">
+      <c r="S15" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">No</t>
         </is>
       </c>
-      <c r="T15" s="81" t="inlineStr">
+      <c r="T15" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="U15" s="81" t="inlineStr">
+      <c r="U15" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="V15" s="81" t="inlineStr">
+      <c r="V15" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="W15" s="81" t="inlineStr">
+      <c r="W15" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="X15" s="83" t="inlineStr">
+      <c r="X15" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="Y15" s="81" t="inlineStr">
+      <c r="Y15" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="Z15" s="83" t="inlineStr">
+      <c r="Z15" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="AA15" s="83" t="inlineStr">
+      <c r="AA15" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">PeiPYHsu</t>
         </is>
       </c>
-      <c r="AB15" s="81"/>
-      <c r="AC15" s="81"/>
-      <c r="AD15" s="81"/>
-      <c r="AE15" s="81"/>
-      <c r="AF15" s="81"/>
-      <c r="AG15" s="81"/>
-      <c r="AH15" s="83" t="inlineStr">
+      <c r="AB15" s="178"/>
+      <c r="AC15" s="178"/>
+      <c r="AD15" s="178"/>
+      <c r="AE15" s="178"/>
+      <c r="AF15" s="178"/>
+      <c r="AG15" s="178"/>
+      <c r="AH15" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">source: 037 SWE1-CertProvider-003 Requirement Description and Verification Criteria
 Polarion: NRL-349386
@@ -8807,40 +8830,40 @@
       </c>
     </row>
     <row r="16" spans="1:34">
-      <c r="A16" s="87"/>
-      <c r="B16" s="81" t="str">
+      <c r="A16" s="182"/>
+      <c r="B16" s="178" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="C16" s="82"/>
-      <c r="D16" s="81" t="inlineStr">
+      <c r="C16" s="179"/>
+      <c r="D16" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">SWE1-CertProvider-004</t>
         </is>
       </c>
-      <c r="E16" s="81"/>
-      <c r="F16" s="81" t="inlineStr">
+      <c r="E16" s="178"/>
+      <c r="F16" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NR1L-CP-007</t>
         </is>
       </c>
-      <c r="G16" s="81" t="inlineStr">
+      <c r="G16" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">Cert Provider</t>
         </is>
       </c>
-      <c r="H16" s="81" t="inlineStr">
+      <c r="H16" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">Revocation</t>
         </is>
       </c>
-      <c r="I16" s="81" t="inlineStr">
+      <c r="I16" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">For non-ECU verification scenarios (e.g., SAM, FOTA, Second Party APKs), the system shall perform revocation checks using Certificate Revocation Lists (CRL) preinstalled in the secure storage of the /odm partition.
 (certificate listed in the local revocation list; certificate is rejected)</t>
         </is>
       </c>
-      <c r="J16" s="81" t="inlineStr">
+      <c r="J16" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. DUT is connected via ADB with root permission (Dev/Eng build)
 2. Test runner CertProviderAndroidInstrumentalTest.apk is installed
@@ -8848,12 +8871,12 @@
 4. Certificate assets are available under SecurityAssets/oem-certs/cert-provider/</t>
         </is>
       </c>
-      <c r="K16" s="81" t="inlineStr">
+      <c r="K16" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NA</t>
         </is>
       </c>
-      <c r="L16" s="81" t="inlineStr">
+      <c r="L16" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. Confirm the content of /odm/etc/cert_store on the DUT
 $ adb shell ls -l /odm/etc/cert_store
@@ -8861,85 +8884,85 @@
 $ &lt;command provided by RD (X-e)&gt;</t>
         </is>
       </c>
-      <c r="M16" s="81" t="inlineStr">
+      <c r="M16" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. The adb shell ls -l /odm/etc/cert_store output lists "CRL.r0"
 2. &lt;log keyword provided by RD (X-h)&gt;</t>
         </is>
       </c>
-      <c r="N16" s="81" t="inlineStr">
+      <c r="N16" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-004</t>
         </is>
       </c>
-      <c r="O16" s="81" t="inlineStr">
+      <c r="O16" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NEW</t>
         </is>
       </c>
-      <c r="P16" s="81" t="inlineStr">
+      <c r="P16" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">P0</t>
         </is>
       </c>
-      <c r="Q16" s="81"/>
-      <c r="R16" s="81" t="inlineStr">
+      <c r="Q16" s="178"/>
+      <c r="R16" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">負向測試 (Negative / Invalid)</t>
         </is>
       </c>
-      <c r="S16" s="81" t="inlineStr">
+      <c r="S16" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">No</t>
         </is>
       </c>
-      <c r="T16" s="81" t="inlineStr">
+      <c r="T16" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="U16" s="81" t="inlineStr">
+      <c r="U16" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="V16" s="81" t="inlineStr">
+      <c r="V16" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="W16" s="81" t="inlineStr">
+      <c r="W16" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="X16" s="83" t="inlineStr">
+      <c r="X16" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="Y16" s="81" t="inlineStr">
+      <c r="Y16" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="Z16" s="83" t="inlineStr">
+      <c r="Z16" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="AA16" s="83" t="inlineStr">
+      <c r="AA16" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">PeiPYHsu</t>
         </is>
       </c>
-      <c r="AB16" s="81"/>
-      <c r="AC16" s="81"/>
-      <c r="AD16" s="81"/>
-      <c r="AE16" s="81"/>
-      <c r="AF16" s="81"/>
-      <c r="AG16" s="81"/>
-      <c r="AH16" s="83" t="inlineStr">
+      <c r="AB16" s="178"/>
+      <c r="AC16" s="178"/>
+      <c r="AD16" s="178"/>
+      <c r="AE16" s="178"/>
+      <c r="AF16" s="178"/>
+      <c r="AG16" s="178"/>
+      <c r="AH16" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">source: 037 SWE1-CertProvider-004 Requirement Description and Verification Criteria
 Polarion: NRL-349387
@@ -8948,7 +8971,8 @@
 asset: X-e — 2. PENDING: X-e revoked certificate + trigger
 asset: X-h — 2. PENDING: X-h log keyword
 conflict: 529/383/532/539 — DCL not deployed; unresolved per CCVR Mapping notes row 10
-scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)</t>
+scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)
+L0 chain path per CCVR note 20260915: /odm/etc/cert_store/ecu_chain — confirm (A-SEC-16)</t>
         </is>
       </c>
     </row>
@@ -9094,135 +9118,135 @@
       </c>
     </row>
     <row r="18" spans="1:34">
-      <c r="A18" s="87"/>
-      <c r="B18" s="81" t="str">
+      <c r="A18" s="182"/>
+      <c r="B18" s="178" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="C18" s="82"/>
-      <c r="D18" s="81" t="inlineStr">
+      <c r="C18" s="179"/>
+      <c r="D18" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">SWE1-CertProvider-005</t>
         </is>
       </c>
-      <c r="E18" s="81"/>
-      <c r="F18" s="81" t="inlineStr">
+      <c r="E18" s="178"/>
+      <c r="F18" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NR1L-CP-009</t>
         </is>
       </c>
-      <c r="G18" s="81" t="inlineStr">
+      <c r="G18" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">Cert Provider</t>
         </is>
       </c>
-      <c r="H18" s="81" t="inlineStr">
+      <c r="H18" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">Revocation</t>
         </is>
       </c>
-      <c r="I18" s="81" t="inlineStr">
+      <c r="I18" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">For ECU verification scenarios, the system shall dynamically retrieve the CRL from the Distribution Point (CDP) URL(s) defined within the target certificate.
 (certificate revoked at the distribution point; certificate is rejected)</t>
         </is>
       </c>
-      <c r="J18" s="81" t="inlineStr">
+      <c r="J18" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. DUT is connected via ADB with root permission (Dev/Eng build)
 2. The DUT has network access
 3. An ECU certificate carrying a valid revocation distribution point is available</t>
         </is>
       </c>
-      <c r="K18" s="81" t="inlineStr">
+      <c r="K18" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NA</t>
         </is>
       </c>
-      <c r="L18" s="81" t="inlineStr">
+      <c r="L18" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. &lt;DUT-side trigger for revoked certificate at the distribution point provided by RD (X-e)&gt;
 $ &lt;command provided by RD (X-e)&gt;</t>
         </is>
       </c>
-      <c r="M18" s="81" t="inlineStr">
+      <c r="M18" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. &lt;log keyword provided by RD (X-h)&gt;</t>
         </is>
       </c>
-      <c r="N18" s="81" t="inlineStr">
+      <c r="N18" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-005</t>
         </is>
       </c>
-      <c r="O18" s="81" t="inlineStr">
+      <c r="O18" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NEW</t>
         </is>
       </c>
-      <c r="P18" s="81" t="inlineStr">
+      <c r="P18" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">P0</t>
         </is>
       </c>
-      <c r="Q18" s="81"/>
-      <c r="R18" s="81" t="inlineStr">
+      <c r="Q18" s="178"/>
+      <c r="R18" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">負向測試 (Negative / Invalid)</t>
         </is>
       </c>
-      <c r="S18" s="81" t="inlineStr">
+      <c r="S18" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">No</t>
         </is>
       </c>
-      <c r="T18" s="81" t="inlineStr">
+      <c r="T18" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="U18" s="81" t="inlineStr">
+      <c r="U18" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="V18" s="81" t="inlineStr">
+      <c r="V18" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="W18" s="81" t="inlineStr">
+      <c r="W18" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="X18" s="83" t="inlineStr">
+      <c r="X18" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="Y18" s="81" t="inlineStr">
+      <c r="Y18" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="Z18" s="83" t="inlineStr">
+      <c r="Z18" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="AA18" s="83" t="inlineStr">
+      <c r="AA18" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">PeiPYHsu</t>
         </is>
       </c>
-      <c r="AB18" s="81"/>
-      <c r="AC18" s="81"/>
-      <c r="AD18" s="81"/>
-      <c r="AE18" s="81"/>
-      <c r="AF18" s="81"/>
-      <c r="AG18" s="81"/>
-      <c r="AH18" s="83" t="inlineStr">
+      <c r="AB18" s="178"/>
+      <c r="AC18" s="178"/>
+      <c r="AD18" s="178"/>
+      <c r="AE18" s="178"/>
+      <c r="AF18" s="178"/>
+      <c r="AG18" s="178"/>
+      <c r="AH18" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">source: 037 SWE1-CertProvider-005 Requirement Description and Verification Criteria
 Polarion: NRL-349388
@@ -9371,7 +9395,8 @@
 sibling axis: storage side effect; rule 1 of SEC-04 4.2
 channel_feasible: Y/Y
 conflict: 529/383/532/539 — DCL not deployed; unresolved per CCVR Mapping notes row 10
-scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)</t>
+scope: service-level validation; reprogramming rejection owned by SWDL (CCVR Cert Val CS.98 rationale)
+L0 chain path per CCVR note 20260915: /odm/etc/cert_store/ecu_chain — confirm (A-SEC-16)</t>
         </is>
       </c>
     </row>
@@ -10066,57 +10091,58 @@
 Polarion: NRL-349390
 sibling axis: store presence; rule 1 of SEC-04 4.2
 channel_feasible: Y/Y
-conflict: 543/546 vs 226; 517 vs 520 — root &amp; CA lifecycle; unresolved per CCVR Mapping notes row 12</t>
+conflict: 543/546 vs 226; 517 vs 520 — root &amp; CA lifecycle; unresolved per CCVR Mapping notes row 12
+L0 chain path per CCVR note 20260915: /odm/etc/cert_store/ecu_chain — confirm (A-SEC-16)</t>
         </is>
       </c>
     </row>
     <row r="25" spans="1:34">
-      <c r="A25" s="87"/>
-      <c r="B25" s="81" t="str">
+      <c r="A25" s="182"/>
+      <c r="B25" s="178" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="C25" s="82"/>
-      <c r="D25" s="81" t="inlineStr">
+      <c r="C25" s="179"/>
+      <c r="D25" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">SWE1-CertProvider-007</t>
         </is>
       </c>
-      <c r="E25" s="81"/>
-      <c r="F25" s="81" t="inlineStr">
+      <c r="E25" s="178"/>
+      <c r="F25" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NR1L-CP-016</t>
         </is>
       </c>
-      <c r="G25" s="81" t="inlineStr">
+      <c r="G25" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">Cert Provider</t>
         </is>
       </c>
-      <c r="H25" s="81" t="inlineStr">
+      <c r="H25" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">Trust Store</t>
         </is>
       </c>
-      <c r="I25" s="81" t="inlineStr">
+      <c r="I25" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">The trusted root and intermediate certificates shall be stored in a persistent, read-only partition that is isolated from user operations.
 (trusted certificate chain survives a factory reset and still verifies a leaf)</t>
         </is>
       </c>
-      <c r="J25" s="81" t="inlineStr">
+      <c r="J25" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. DUT is connected via ADB with root permission (Dev/Eng build)
 2. Test runner CertProviderAndroidInstrumentalTest.apk is installed
 3. Certificate assets are available under SecurityAssets/oem-certs/cert-provider/</t>
         </is>
       </c>
-      <c r="K25" s="81" t="inlineStr">
+      <c r="K25" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NA</t>
         </is>
       </c>
-      <c r="L25" s="81" t="inlineStr">
+      <c r="L25" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. Confirm the content of /odm/etc/cert_store on the DUT
 $ adb shell ls -l /odm/etc/cert_store
@@ -10126,86 +10152,86 @@
 $ &lt;command provided by RD (X-e)&gt;</t>
         </is>
       </c>
-      <c r="M25" s="81" t="inlineStr">
+      <c r="M25" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. The adb shell ls -l /odm/etc/cert_store output lists the trusted certificate chain files
 2. The openssl command prints "SAMcert.pem: OK" on stdout
 3. &lt;log keyword provided by RD (X-h)&gt;</t>
         </is>
       </c>
-      <c r="N25" s="81" t="inlineStr">
+      <c r="N25" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-007</t>
         </is>
       </c>
-      <c r="O25" s="81" t="inlineStr">
+      <c r="O25" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NEW</t>
         </is>
       </c>
-      <c r="P25" s="81" t="inlineStr">
+      <c r="P25" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">P1</t>
         </is>
       </c>
-      <c r="Q25" s="81"/>
-      <c r="R25" s="81" t="inlineStr">
+      <c r="Q25" s="178"/>
+      <c r="R25" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">功能測試 (Functional based ; no specific technique)</t>
         </is>
       </c>
-      <c r="S25" s="81" t="inlineStr">
+      <c r="S25" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">No</t>
         </is>
       </c>
-      <c r="T25" s="81" t="inlineStr">
+      <c r="T25" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="U25" s="81" t="inlineStr">
+      <c r="U25" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="V25" s="81" t="inlineStr">
+      <c r="V25" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="W25" s="81" t="inlineStr">
+      <c r="W25" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="X25" s="83" t="inlineStr">
+      <c r="X25" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="Y25" s="81" t="inlineStr">
+      <c r="Y25" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="Z25" s="83" t="inlineStr">
+      <c r="Z25" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="AA25" s="83" t="inlineStr">
+      <c r="AA25" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">PeiPYHsu</t>
         </is>
       </c>
-      <c r="AB25" s="81"/>
-      <c r="AC25" s="81"/>
-      <c r="AD25" s="81"/>
-      <c r="AE25" s="81"/>
-      <c r="AF25" s="81"/>
-      <c r="AG25" s="81"/>
-      <c r="AH25" s="83" t="inlineStr">
+      <c r="AB25" s="178"/>
+      <c r="AC25" s="178"/>
+      <c r="AD25" s="178"/>
+      <c r="AE25" s="178"/>
+      <c r="AF25" s="178"/>
+      <c r="AG25" s="178"/>
+      <c r="AH25" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">source: 037 SWE1-CertProvider-007 Requirement Description and Verification Criteria
 Polarion: NRL-349390
@@ -10213,45 +10239,46 @@
 channel_feasible: Y/Y
 asset: X-e — 3. PENDING: X-e valid leaf certificate + trigger
 asset: X-h — 3. PENDING: X-h log keyword
-conflict: 543/546 vs 226; 517 vs 520 — root &amp; CA lifecycle; unresolved per CCVR Mapping notes row 12</t>
+conflict: 543/546 vs 226; 517 vs 520 — root &amp; CA lifecycle; unresolved per CCVR Mapping notes row 12
+L0 chain path per CCVR note 20260915: /odm/etc/cert_store/ecu_chain — confirm (A-SEC-16)</t>
         </is>
       </c>
     </row>
     <row r="26" spans="1:34">
-      <c r="A26" s="87"/>
-      <c r="B26" s="81" t="str">
+      <c r="A26" s="182"/>
+      <c r="B26" s="178" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="C26" s="82"/>
-      <c r="D26" s="81" t="inlineStr">
+      <c r="C26" s="179"/>
+      <c r="D26" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">SWE1-CertProvider-008</t>
         </is>
       </c>
-      <c r="E26" s="81"/>
-      <c r="F26" s="81" t="inlineStr">
+      <c r="E26" s="178"/>
+      <c r="F26" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NR1L-CP-017</t>
         </is>
       </c>
-      <c r="G26" s="81" t="inlineStr">
+      <c r="G26" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">Cert Provider</t>
         </is>
       </c>
-      <c r="H26" s="81" t="inlineStr">
+      <c r="H26" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">Client Interface</t>
         </is>
       </c>
-      <c r="I26" s="81" t="inlineStr">
+      <c r="I26" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">The Cert Provider feature shall provide standardized client interfaces to support both Java and Native clients.
 (Java client invokes the Binder interface for certificate validation (document review + log observation))</t>
         </is>
       </c>
-      <c r="J26" s="81" t="inlineStr">
+      <c r="J26" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. DUT is connected via ADB with root permission (Dev/Eng build)
 2. Test runner CertProviderAndroidInstrumentalTest.apk is installed
@@ -10259,12 +10286,12 @@
 4. Access to the RD build environment for Cert Provider is granted</t>
         </is>
       </c>
-      <c r="K26" s="81" t="inlineStr">
+      <c r="K26" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NA</t>
         </is>
       </c>
-      <c r="L26" s="81" t="inlineStr">
+      <c r="L26" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. &lt;obtain the source code and dependency graph of the Java clients per RD&gt;
 2. Review the source code and dependency graph of the Java clients against "Verify they link against and invoke the CertProvider Binder interface for certificate validation"
@@ -10272,86 +10299,86 @@
 $ adb logcat -s Logdog</t>
         </is>
       </c>
-      <c r="M26" s="81" t="inlineStr">
+      <c r="M26" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. The source code and dependency graph of the Java clients are available for review
 2. The source code and dependency graph of the Java clients satisfy "Verify they link against and invoke the CertProvider Binder interface for certificate validation"
 3. &lt;log keyword provided by RD (X-h)&gt;</t>
         </is>
       </c>
-      <c r="N26" s="81" t="inlineStr">
+      <c r="N26" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-008</t>
         </is>
       </c>
-      <c r="O26" s="81" t="inlineStr">
+      <c r="O26" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NEW</t>
         </is>
       </c>
-      <c r="P26" s="81" t="inlineStr">
+      <c r="P26" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">P1</t>
         </is>
       </c>
-      <c r="Q26" s="81"/>
-      <c r="R26" s="81" t="inlineStr">
+      <c r="Q26" s="178"/>
+      <c r="R26" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">功能測試 (Functional based ; no specific technique)</t>
         </is>
       </c>
-      <c r="S26" s="81" t="inlineStr">
+      <c r="S26" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">No</t>
         </is>
       </c>
-      <c r="T26" s="81" t="inlineStr">
+      <c r="T26" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="U26" s="81" t="inlineStr">
+      <c r="U26" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="V26" s="81" t="inlineStr">
+      <c r="V26" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="W26" s="81" t="inlineStr">
+      <c r="W26" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="X26" s="83" t="inlineStr">
+      <c r="X26" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="Y26" s="81" t="inlineStr">
+      <c r="Y26" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="Z26" s="83" t="inlineStr">
+      <c r="Z26" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="AA26" s="83" t="inlineStr">
+      <c r="AA26" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">PeiPYHsu</t>
         </is>
       </c>
-      <c r="AB26" s="81"/>
-      <c r="AC26" s="81"/>
-      <c r="AD26" s="81"/>
-      <c r="AE26" s="81"/>
-      <c r="AF26" s="81"/>
-      <c r="AG26" s="81"/>
-      <c r="AH26" s="83" t="inlineStr">
+      <c r="AB26" s="178"/>
+      <c r="AC26" s="178"/>
+      <c r="AD26" s="178"/>
+      <c r="AE26" s="178"/>
+      <c r="AF26" s="178"/>
+      <c r="AG26" s="178"/>
+      <c r="AH26" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">verification: document review (R-SEC20)
 Polarion: NRL-349391
@@ -10364,40 +10391,40 @@
       </c>
     </row>
     <row r="27" spans="1:34">
-      <c r="A27" s="87"/>
-      <c r="B27" s="81" t="str">
+      <c r="A27" s="182"/>
+      <c r="B27" s="178" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="C27" s="82"/>
-      <c r="D27" s="81" t="inlineStr">
+      <c r="C27" s="179"/>
+      <c r="D27" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">SWE1-CertProvider-008</t>
         </is>
       </c>
-      <c r="E27" s="81"/>
-      <c r="F27" s="81" t="inlineStr">
+      <c r="E27" s="178"/>
+      <c r="F27" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NR1L-CP-018</t>
         </is>
       </c>
-      <c r="G27" s="81" t="inlineStr">
+      <c r="G27" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">Cert Provider</t>
         </is>
       </c>
-      <c r="H27" s="81" t="inlineStr">
+      <c r="H27" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">Client Interface</t>
         </is>
       </c>
-      <c r="I27" s="81" t="inlineStr">
+      <c r="I27" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">The Cert Provider feature shall provide standardized client interfaces to support both Java and Native clients.
 (Native client uses the libCertProvider C++ API for leaf verification (document review + log observation))</t>
         </is>
       </c>
-      <c r="J27" s="81" t="inlineStr">
+      <c r="J27" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. DUT is connected via ADB with root permission (Dev/Eng build)
 2. Test runner CertProviderAndroidInstrumentalTest.apk is installed
@@ -10405,12 +10432,12 @@
 4. Access to the RD build environment for Cert Provider is granted</t>
         </is>
       </c>
-      <c r="K27" s="81" t="inlineStr">
+      <c r="K27" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NA</t>
         </is>
       </c>
-      <c r="L27" s="81" t="inlineStr">
+      <c r="L27" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. &lt;obtain the Native client implementations per RD&gt;
 2. Review the Native client implementations against "Verify they utilize the libCertProvider C++ API for leaf certificate verification"
@@ -10418,86 +10445,86 @@
 $ adb logcat -s Logdog</t>
         </is>
       </c>
-      <c r="M27" s="81" t="inlineStr">
+      <c r="M27" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. The Native client implementations are available for review
 2. The Native client implementations satisfy "Verify they utilize the libCertProvider C++ API for leaf certificate verification"
 3. &lt;log keyword provided by RD (X-h)&gt;</t>
         </is>
       </c>
-      <c r="N27" s="81" t="inlineStr">
+      <c r="N27" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-008</t>
         </is>
       </c>
-      <c r="O27" s="81" t="inlineStr">
+      <c r="O27" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NEW</t>
         </is>
       </c>
-      <c r="P27" s="81" t="inlineStr">
+      <c r="P27" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">P1</t>
         </is>
       </c>
-      <c r="Q27" s="81"/>
-      <c r="R27" s="81" t="inlineStr">
+      <c r="Q27" s="178"/>
+      <c r="R27" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">功能測試 (Functional based ; no specific technique)</t>
         </is>
       </c>
-      <c r="S27" s="81" t="inlineStr">
+      <c r="S27" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">No</t>
         </is>
       </c>
-      <c r="T27" s="81" t="inlineStr">
+      <c r="T27" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="U27" s="81" t="inlineStr">
+      <c r="U27" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="V27" s="81" t="inlineStr">
+      <c r="V27" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="W27" s="81" t="inlineStr">
+      <c r="W27" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="X27" s="83" t="inlineStr">
+      <c r="X27" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="Y27" s="81" t="inlineStr">
+      <c r="Y27" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="Z27" s="83" t="inlineStr">
+      <c r="Z27" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="AA27" s="83" t="inlineStr">
+      <c r="AA27" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">PeiPYHsu</t>
         </is>
       </c>
-      <c r="AB27" s="81"/>
-      <c r="AC27" s="81"/>
-      <c r="AD27" s="81"/>
-      <c r="AE27" s="81"/>
-      <c r="AF27" s="81"/>
-      <c r="AG27" s="81"/>
-      <c r="AH27" s="83" t="inlineStr">
+      <c r="AB27" s="178"/>
+      <c r="AC27" s="178"/>
+      <c r="AD27" s="178"/>
+      <c r="AE27" s="178"/>
+      <c r="AF27" s="178"/>
+      <c r="AG27" s="178"/>
+      <c r="AH27" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">verification: document review (R-SEC20)
 Polarion: NRL-349391
@@ -10647,57 +10674,58 @@
 Polarion: NRL-349392
 sibling axis: configuration version; rule 1,2 of SEC-04 4.2
 channel_feasible: Y/Y
-conflict: 543/546 vs 226; 517 vs 520 — root &amp; CA lifecycle; unresolved per CCVR Mapping notes row 12</t>
+conflict: 543/546 vs 226; 517 vs 520 — root &amp; CA lifecycle; unresolved per CCVR Mapping notes row 12
+L0 chain path per CCVR note 20260915: /odm/etc/cert_store/ecu_chain — confirm (A-SEC-16)</t>
         </is>
       </c>
     </row>
     <row r="29" spans="1:34">
-      <c r="A29" s="87"/>
-      <c r="B29" s="81" t="str">
+      <c r="A29" s="182"/>
+      <c r="B29" s="178" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="C29" s="82"/>
-      <c r="D29" s="81" t="inlineStr">
+      <c r="C29" s="179"/>
+      <c r="D29" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">SWE1-CertProvider-009</t>
         </is>
       </c>
-      <c r="E29" s="81"/>
-      <c r="F29" s="81" t="inlineStr">
+      <c r="E29" s="178"/>
+      <c r="F29" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NR1L-CP-020</t>
         </is>
       </c>
-      <c r="G29" s="81" t="inlineStr">
+      <c r="G29" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">Cert Provider</t>
         </is>
       </c>
-      <c r="H29" s="81" t="inlineStr">
+      <c r="H29" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">Trust Store</t>
         </is>
       </c>
-      <c r="I29" s="81" t="inlineStr">
+      <c r="I29" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">The Cert Provider feature shall be able to switch verification configurations between the development version software and the product version software.
 (Product configuration; the matching certificate chain is deployed)</t>
         </is>
       </c>
-      <c r="J29" s="81" t="inlineStr">
+      <c r="J29" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. DUT is connected via ADB with root permission (Dev/Eng build)
 2. Test runner CertProviderAndroidInstrumentalTest.apk is installed
 3. Certificate assets are available under SecurityAssets/oem-certs/cert-provider/</t>
         </is>
       </c>
-      <c r="K29" s="81" t="inlineStr">
+      <c r="K29" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NA</t>
         </is>
       </c>
-      <c r="L29" s="81" t="inlineStr">
+      <c r="L29" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. Confirm the content of /odm/etc/cert_store on the DUT
 $ adb shell ls -l /odm/etc/cert_store
@@ -10705,85 +10733,85 @@
 $ &lt;command provided by STLA (X-c)&gt;</t>
         </is>
       </c>
-      <c r="M29" s="81" t="inlineStr">
+      <c r="M29" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. The adb shell ls -l /odm/etc/cert_store output lists the Product certificate chain
 2. &lt;log keyword provided by RD (X-h)&gt;</t>
         </is>
       </c>
-      <c r="N29" s="81" t="inlineStr">
+      <c r="N29" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-009</t>
         </is>
       </c>
-      <c r="O29" s="81" t="inlineStr">
+      <c r="O29" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NEW</t>
         </is>
       </c>
-      <c r="P29" s="81" t="inlineStr">
+      <c r="P29" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">P1</t>
         </is>
       </c>
-      <c r="Q29" s="81"/>
-      <c r="R29" s="81" t="inlineStr">
+      <c r="Q29" s="178"/>
+      <c r="R29" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">功能測試 (Functional based ; no specific technique)</t>
         </is>
       </c>
-      <c r="S29" s="81" t="inlineStr">
+      <c r="S29" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">No</t>
         </is>
       </c>
-      <c r="T29" s="81" t="inlineStr">
+      <c r="T29" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="U29" s="81" t="inlineStr">
+      <c r="U29" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="V29" s="81" t="inlineStr">
+      <c r="V29" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="W29" s="81" t="inlineStr">
+      <c r="W29" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="X29" s="83" t="inlineStr">
+      <c r="X29" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="Y29" s="81" t="inlineStr">
+      <c r="Y29" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="Z29" s="83" t="inlineStr">
+      <c r="Z29" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="AA29" s="83" t="inlineStr">
+      <c r="AA29" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">PeiPYHsu</t>
         </is>
       </c>
-      <c r="AB29" s="81"/>
-      <c r="AC29" s="81"/>
-      <c r="AD29" s="81"/>
-      <c r="AE29" s="81"/>
-      <c r="AF29" s="81"/>
-      <c r="AG29" s="81"/>
-      <c r="AH29" s="83" t="inlineStr">
+      <c r="AB29" s="178"/>
+      <c r="AC29" s="178"/>
+      <c r="AD29" s="178"/>
+      <c r="AE29" s="178"/>
+      <c r="AF29" s="178"/>
+      <c r="AG29" s="178"/>
+      <c r="AH29" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">source: 037 SWE1-CertProvider-009 Requirement Description and Verification Criteria
 Polarion: NRL-349392
@@ -10791,7 +10819,8 @@
 channel_feasible: Y/Y
 asset: X-c — 2. PENDING: X-c NR1L production certificate + trigger
 asset: X-h — 2. PENDING: X-h log keyword
-conflict: 543/546 vs 226; 517 vs 520 — root &amp; CA lifecycle; unresolved per CCVR Mapping notes row 12</t>
+conflict: 543/546 vs 226; 517 vs 520 — root &amp; CA lifecycle; unresolved per CCVR Mapping notes row 12
+L0 chain path per CCVR note 20260915: /odm/etc/cert_store/ecu_chain — confirm (A-SEC-16)</t>
         </is>
       </c>
     </row>
@@ -10938,52 +10967,52 @@
       </c>
     </row>
     <row r="31" spans="1:34">
-      <c r="A31" s="87"/>
-      <c r="B31" s="81" t="str">
+      <c r="A31" s="182"/>
+      <c r="B31" s="178" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="C31" s="82"/>
-      <c r="D31" s="81" t="inlineStr">
+      <c r="C31" s="179"/>
+      <c r="D31" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">SWE1-CertProvider-011</t>
         </is>
       </c>
-      <c r="E31" s="81"/>
-      <c r="F31" s="81" t="inlineStr">
+      <c r="E31" s="178"/>
+      <c r="F31" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NR1L-CP-022</t>
         </is>
       </c>
-      <c r="G31" s="81" t="inlineStr">
+      <c r="G31" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">Cert Provider</t>
         </is>
       </c>
-      <c r="H31" s="81" t="inlineStr">
+      <c r="H31" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">Field Matching</t>
         </is>
       </c>
-      <c r="I31" s="81" t="inlineStr">
+      <c r="I31" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">The Cert Provider feature shall support the validation of project-specific critical extensions within the leaf certificate.
 (extension value is the project identifier; certificate is accepted)</t>
         </is>
       </c>
-      <c r="J31" s="81" t="inlineStr">
+      <c r="J31" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. DUT is connected via ADB with root permission (Dev/Eng build)
 2. Test runner CertProviderAndroidInstrumentalTest.apk is installed
 3. Certificate assets are available under SecurityAssets/oem-certs/cert-provider/</t>
         </is>
       </c>
-      <c r="K31" s="81" t="inlineStr">
+      <c r="K31" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NA</t>
         </is>
       </c>
-      <c r="L31" s="81" t="inlineStr">
+      <c r="L31" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. Read the certificate extensions of the certificate on the host
 $ openssl x509 -in leaf.crt -text
@@ -10993,86 +11022,86 @@
 $ &lt;command provided by RD (X-e)&gt;</t>
         </is>
       </c>
-      <c r="M31" s="81" t="inlineStr">
+      <c r="M31" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. The openssl x509 output shows "X509v3 Certificate Policies: critical" and a "Policy:" line with the OID 1.3.6.1.4.1.57872.&lt;…&gt;
 2. The openssl command prints "SAMcert.pem: OK" on stdout
 3. &lt;log keyword provided by RD (X-h)&gt;</t>
         </is>
       </c>
-      <c r="N31" s="81" t="inlineStr">
+      <c r="N31" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-011</t>
         </is>
       </c>
-      <c r="O31" s="81" t="inlineStr">
+      <c r="O31" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NEW</t>
         </is>
       </c>
-      <c r="P31" s="81" t="inlineStr">
+      <c r="P31" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">P1</t>
         </is>
       </c>
-      <c r="Q31" s="81"/>
-      <c r="R31" s="81" t="inlineStr">
+      <c r="Q31" s="178"/>
+      <c r="R31" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">功能測試 (Functional based ; no specific technique)</t>
         </is>
       </c>
-      <c r="S31" s="81" t="inlineStr">
+      <c r="S31" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">No</t>
         </is>
       </c>
-      <c r="T31" s="81" t="inlineStr">
+      <c r="T31" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="U31" s="81" t="inlineStr">
+      <c r="U31" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="V31" s="81" t="inlineStr">
+      <c r="V31" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="W31" s="81" t="inlineStr">
+      <c r="W31" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="X31" s="83" t="inlineStr">
+      <c r="X31" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="Y31" s="81" t="inlineStr">
+      <c r="Y31" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="Z31" s="83" t="inlineStr">
+      <c r="Z31" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="AA31" s="83" t="inlineStr">
+      <c r="AA31" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">PeiPYHsu</t>
         </is>
       </c>
-      <c r="AB31" s="81"/>
-      <c r="AC31" s="81"/>
-      <c r="AD31" s="81"/>
-      <c r="AE31" s="81"/>
-      <c r="AF31" s="81"/>
-      <c r="AG31" s="81"/>
-      <c r="AH31" s="83" t="inlineStr">
+      <c r="AB31" s="178"/>
+      <c r="AC31" s="178"/>
+      <c r="AD31" s="178"/>
+      <c r="AE31" s="178"/>
+      <c r="AF31" s="178"/>
+      <c r="AG31" s="178"/>
+      <c r="AH31" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">source: 037 SWE1-CertProvider-011 Requirement Description and Verification Criteria
 Polarion: NRL-349394
@@ -11084,52 +11113,52 @@
       </c>
     </row>
     <row r="32" spans="1:34">
-      <c r="A32" s="87"/>
-      <c r="B32" s="81" t="str">
+      <c r="A32" s="182"/>
+      <c r="B32" s="178" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="C32" s="82"/>
-      <c r="D32" s="81" t="inlineStr">
+      <c r="C32" s="179"/>
+      <c r="D32" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">SWE1-CertProvider-011</t>
         </is>
       </c>
-      <c r="E32" s="81"/>
-      <c r="F32" s="81" t="inlineStr">
+      <c r="E32" s="178"/>
+      <c r="F32" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NR1L-CP-023</t>
         </is>
       </c>
-      <c r="G32" s="81" t="inlineStr">
+      <c r="G32" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">Cert Provider</t>
         </is>
       </c>
-      <c r="H32" s="81" t="inlineStr">
+      <c r="H32" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">Field Matching</t>
         </is>
       </c>
-      <c r="I32" s="81" t="inlineStr">
+      <c r="I32" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">The Cert Provider feature shall support the validation of project-specific critical extensions within the leaf certificate.
 (extension value is incorrect or missing; certificate is rejected)</t>
         </is>
       </c>
-      <c r="J32" s="81" t="inlineStr">
+      <c r="J32" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. DUT is connected via ADB with root permission (Dev/Eng build)
 2. Test runner CertProviderAndroidInstrumentalTest.apk is installed
 3. Certificate assets are available under SecurityAssets/oem-certs/cert-provider/</t>
         </is>
       </c>
-      <c r="K32" s="81" t="inlineStr">
+      <c r="K32" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NA</t>
         </is>
       </c>
-      <c r="L32" s="81" t="inlineStr">
+      <c r="L32" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. Read the certificate extensions of the certificate on the host
 $ openssl x509 -in leaf.crt -text
@@ -11137,85 +11166,85 @@
 $ &lt;command provided by RD (X-e)&gt;</t>
         </is>
       </c>
-      <c r="M32" s="81" t="inlineStr">
+      <c r="M32" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1. The openssl x509 output shows no "X509v3 Certificate Policies: critical" line, or a "Policy:" line whose OID is not 1.3.6.1.4.1.57872.&lt;…&gt;
 2. &lt;log keyword provided by RD (X-h)&gt;</t>
         </is>
       </c>
-      <c r="N32" s="81" t="inlineStr">
+      <c r="N32" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">SWE1-CertProvider-SWE1R1-V1.0_SWE1-CertProvider-011</t>
         </is>
       </c>
-      <c r="O32" s="81" t="inlineStr">
+      <c r="O32" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">NEW</t>
         </is>
       </c>
-      <c r="P32" s="81" t="inlineStr">
+      <c r="P32" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">P1</t>
         </is>
       </c>
-      <c r="Q32" s="81"/>
-      <c r="R32" s="81" t="inlineStr">
+      <c r="Q32" s="178"/>
+      <c r="R32" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">負向測試 (Negative / Invalid)</t>
         </is>
       </c>
-      <c r="S32" s="81" t="inlineStr">
+      <c r="S32" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">No</t>
         </is>
       </c>
-      <c r="T32" s="81" t="inlineStr">
+      <c r="T32" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="U32" s="81" t="inlineStr">
+      <c r="U32" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="V32" s="81" t="inlineStr">
+      <c r="V32" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="W32" s="81" t="inlineStr">
+      <c r="W32" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="X32" s="83" t="inlineStr">
+      <c r="X32" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">0</t>
         </is>
       </c>
-      <c r="Y32" s="81" t="inlineStr">
+      <c r="Y32" s="178" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="Z32" s="83" t="inlineStr">
+      <c r="Z32" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">1</t>
         </is>
       </c>
-      <c r="AA32" s="83" t="inlineStr">
+      <c r="AA32" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">PeiPYHsu</t>
         </is>
       </c>
-      <c r="AB32" s="81"/>
-      <c r="AC32" s="81"/>
-      <c r="AD32" s="81"/>
-      <c r="AE32" s="81"/>
-      <c r="AF32" s="81"/>
-      <c r="AG32" s="81"/>
-      <c r="AH32" s="83" t="inlineStr">
+      <c r="AB32" s="178"/>
+      <c r="AC32" s="178"/>
+      <c r="AD32" s="178"/>
+      <c r="AE32" s="178"/>
+      <c r="AF32" s="178"/>
+      <c r="AG32" s="178"/>
+      <c r="AH32" s="180" t="inlineStr">
         <is>
           <t xml:space="preserve">source: 037 SWE1-CertProvider-011 Requirement Description and Verification Criteria
 Polarion: NRL-349394

</xml_diff>